<commit_message>
fix:Mejora en la estructura del codigo + agregado de buenas practicas + agregado de json y xml para los reportes de cucumber
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/DatosPrueba_Admin.xlsx
+++ b/src/test/resources/testData/DatosPrueba_Admin.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="UsuarioDuplicado" sheetId="1" state="visible" r:id="rId1"/>
@@ -30,9 +30,6 @@
     <t>TC-009</t>
   </si>
   <si>
-    <t>ebe</t>
-  </si>
-  <si>
     <t>userRole</t>
   </si>
   <si>
@@ -48,7 +45,7 @@
     <t>confirmPassword</t>
   </si>
   <si>
-    <t xml:space="preserve">que s</t>
+    <t>TC-08</t>
   </si>
   <si>
     <t>Admin</t>
@@ -58,6 +55,9 @@
   </si>
   <si>
     <t>Enabled</t>
+  </si>
+  <si>
+    <t>username123</t>
   </si>
   <si>
     <t>Admin123!</t>
@@ -4822,42 +4822,42 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
       <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>5</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>6</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="6" t="s">
+    </row>
+    <row r="2" ht="21.75" customHeight="1">
+      <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" ht="21.75" customHeight="1">
-      <c r="A2" s="7" t="s">
+      <c r="B2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>12</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>1</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>13</v>

</xml_diff>